<commit_message>
feat(content): add XLOOKUP article visuals
</commit_message>
<xml_diff>
--- a/public/downloads/templates/xlookup-complete-guide.xlsx
+++ b/public/downloads/templates/xlookup-complete-guide.xlsx
@@ -1,15 +1,54 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAE5FA05-DDFF-4067-8320-CF2E4ACD43F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Basic &amp; Errors" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Left Lookup &amp; Spill" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Approximate (Tax)" state="visible" r:id="rId6"/>
+    <sheet name="Basic &amp; Errors" sheetId="1" r:id="rId1"/>
+    <sheet name="Left Lookup &amp; Spill" sheetId="2" r:id="rId2"/>
+    <sheet name="Approximate (Tax)" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -180,25 +219,36 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF6B7280"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <i/>
-      <color rgb="FF6B7280"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -228,10 +278,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -240,9 +291,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -578,9 +631,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -590,7 +643,7 @@
     <col min="7" max="8" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -633,13 +686,15 @@
         <v>10</v>
       </c>
       <c r="G2">
-        <f>XLOOKUP(F2,A2:A7,C2:C7)</f>
-      </c>
-      <c r="H2">
-        <f>XLOOKUP("P999",A2:A7,C2:C7,"Not found")</f>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <f>_xlfn.SINGLE(_xlfn.XLOOKUP(F2,A2:A7,C2:C7))</f>
+        <v>89.99</v>
+      </c>
+      <c r="H2" t="str">
+        <f>_xlfn.SINGLE(_xlfn.XLOOKUP("P999",A2:A7,C2:C7,"Not found"))</f>
+        <v>Not found</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -653,7 +708,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -667,7 +722,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -681,7 +736,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -695,7 +750,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -709,26 +764,26 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>21</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="3" width="13" customWidth="1"/>
@@ -740,7 +795,7 @@
     <col min="9" max="9" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -769,7 +824,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -782,17 +837,25 @@
       <c r="E2" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F2">
-        <f>XLOOKUP(E2,C2:C7,A2:A7)</f>
+      <c r="F2" t="str">
+        <f>_xlfn.SINGLE(_xlfn.XLOOKUP(E2,C2:C7,A2:A7))</f>
+        <v>Ben Ortega</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I2">
-        <f>XLOOKUP(H2,'Basic &amp; Errors'!A2:A7,'Basic &amp; Errors'!B2:D7)</f>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I2" t="str" cm="1">
+        <f t="array" ref="I2:K2">_xlfn.XLOOKUP(H2,'Basic &amp; Errors'!A2:A7,'Basic &amp; Errors'!B2:D7)</f>
+        <v>Monitor Arm</v>
+      </c>
+      <c r="J2">
+        <v>89.99</v>
+      </c>
+      <c r="K2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -803,7 +866,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -814,7 +877,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -825,7 +888,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -836,7 +899,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -847,26 +910,26 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
@@ -875,7 +938,7 @@
     <col min="5" max="5" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>49</v>
       </c>
@@ -902,8 +965,9 @@
       <c r="D2" s="3">
         <v>75000</v>
       </c>
-      <c r="E2">
-        <f>XLOOKUP(D2,A2:A5,B2:B5,,-1)</f>
+      <c r="E2" s="6">
+        <f>_xlfn.XLOOKUP(D2,A2:A5,B2:B5,,-1)</f>
+        <v>0.2</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -930,13 +994,13 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>53</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>